<commit_message>
Sincronizar cambios locales: partida, tienda, asaltos, mazos, misiones, opciones, tablero, iconos y servidor
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/asaltos.xlsx
+++ b/public/resources/asaltos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB38888-AB7A-4FDA-BA50-4A2A3FBD1C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126E3698-6BA0-4854-9058-687E3420D4FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="46">
   <si>
     <t>asalto_ID</t>
   </si>
@@ -90,9 +90,6 @@
     <t>mejora_definitiva</t>
   </si>
   <si>
-    <t>fragmentos</t>
-  </si>
-  <si>
     <t>Grim Knight</t>
   </si>
   <si>
@@ -154,6 +151,18 @@
   </si>
   <si>
     <t>https://i.ibb.co/Jw48W52F/dark-nights-metal-ranking-the-dark-batmans-from-best-to-v0-jb3gszsxps1b1.webp</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
 </sst>
 </file>
@@ -227,7 +236,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -510,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:W7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -521,10 +530,9 @@
     <col min="21" max="21" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="17" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -532,13 +540,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -594,442 +602,421 @@
       <c r="W1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="X1" s="1" t="s">
-        <v>21</v>
-      </c>
     </row>
-    <row r="2" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="E2" s="2">
         <v>6</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" s="3" t="s">
+      <c r="L2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="R2" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="S2" s="2">
         <v>1200</v>
       </c>
       <c r="T2" s="4">
-        <v>0.75</v>
-      </c>
-      <c r="U2" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="V2" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="W2" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="X2" s="2">
-        <v>2</v>
+        <v>50</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="V2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="W2" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E3" s="2">
         <v>7</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="3" t="s">
+      <c r="L3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="R3" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="S3" s="2">
         <v>1200</v>
       </c>
-      <c r="T3" s="4">
-        <v>0.75</v>
-      </c>
-      <c r="U3" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="V3" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="W3" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="X3" s="2">
-        <v>2</v>
+      <c r="T3" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E4" s="2">
         <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" s="3" t="s">
+      <c r="L4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q4" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="R4" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="S4" s="2">
         <v>1200</v>
       </c>
-      <c r="T4" s="4">
-        <v>0.75</v>
-      </c>
-      <c r="U4" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="V4" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="W4" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="X4" s="2">
-        <v>2</v>
+      <c r="T4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="U4" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="V4" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="W4" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E5" s="2">
         <v>7</v>
       </c>
       <c r="F5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I5" s="3" t="s">
+      <c r="L5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="R5" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="S5" s="2">
         <v>1200</v>
       </c>
-      <c r="T5" s="4">
-        <v>0.75</v>
-      </c>
-      <c r="U5" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="V5" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="W5" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="X5" s="2">
-        <v>2</v>
+      <c r="T5" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="V5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="W5" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6" s="2">
         <v>8</v>
       </c>
       <c r="F6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="3" t="s">
+      <c r="L6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q6" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="R6" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="S6" s="2">
         <v>1200</v>
       </c>
-      <c r="T6" s="4">
-        <v>0.75</v>
-      </c>
-      <c r="U6" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="V6" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="W6" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="X6" s="2">
-        <v>2</v>
+      <c r="T6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="U6" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="V6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="W6" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" s="2">
         <v>7</v>
       </c>
       <c r="F7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I7" s="3" t="s">
+      <c r="L7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="O7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="R7" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="S7" s="2">
         <v>1200</v>
       </c>
-      <c r="T7" s="4">
-        <v>0.75</v>
-      </c>
-      <c r="U7" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="V7" s="4">
-        <v>0.25</v>
-      </c>
-      <c r="W7" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="X7" s="2">
-        <v>2</v>
+      <c r="T7" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="U7" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="V7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="W7" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Release 1.2.1: skills, formulas, heal-debuff, shield UI, tienda sync.
Bump version label and packages. Combat skill_power uses formulas and
correct scaling; buff/debuff/bonus_buff ignore table buffs; shop refreshes
offers from Excel during active rotation.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/asaltos.xlsx
+++ b/public/resources/asaltos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126E3698-6BA0-4854-9058-687E3420D4FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01B666A-F980-466C-9D4C-2F8072027561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="47">
   <si>
     <t>asalto_ID</t>
   </si>
@@ -163,13 +163,16 @@
   </si>
   <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>https://images-ext-1.discordapp.net/external/4KzH3137pygQQi3r1ftpAi2LL9alkwXhYMY0R5kb8jA/https/speedforce.org/wp-content/uploads/2011/07/sdcc-flashpoint.jpg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,6 +182,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -222,8 +233,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -236,11 +248,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -661,16 +674,16 @@
       <c r="S2" s="2">
         <v>1200</v>
       </c>
-      <c r="T2" s="4">
+      <c r="T2" s="2">
         <v>50</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="V2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="W2" s="2" t="s">
         <v>45</v>
       </c>
     </row>
@@ -681,7 +694,9 @@
       <c r="B3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="4" t="s">
+        <v>46</v>
+      </c>
       <c r="D3" s="2" t="s">
         <v>32</v>
       </c>
@@ -730,16 +745,16 @@
       <c r="S3" s="2">
         <v>1200</v>
       </c>
-      <c r="T3" s="4" t="s">
+      <c r="T3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U3" s="4" t="s">
+      <c r="U3" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="V3" s="4" t="s">
+      <c r="V3" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="W3" s="4" t="s">
+      <c r="W3" s="2" t="s">
         <v>45</v>
       </c>
     </row>
@@ -799,16 +814,16 @@
       <c r="S4" s="2">
         <v>1200</v>
       </c>
-      <c r="T4" s="4" t="s">
+      <c r="T4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U4" s="4" t="s">
+      <c r="U4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="V4" s="4" t="s">
+      <c r="V4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="W4" s="4" t="s">
+      <c r="W4" s="2" t="s">
         <v>45</v>
       </c>
     </row>
@@ -868,16 +883,16 @@
       <c r="S5" s="2">
         <v>1200</v>
       </c>
-      <c r="T5" s="4" t="s">
+      <c r="T5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U5" s="4" t="s">
+      <c r="U5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="V5" s="4" t="s">
+      <c r="V5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="W5" s="4" t="s">
+      <c r="W5" s="2" t="s">
         <v>45</v>
       </c>
     </row>
@@ -937,16 +952,16 @@
       <c r="S6" s="2">
         <v>1200</v>
       </c>
-      <c r="T6" s="4" t="s">
+      <c r="T6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U6" s="4" t="s">
+      <c r="U6" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="V6" s="4" t="s">
+      <c r="V6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="W6" s="4" t="s">
+      <c r="W6" s="2" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1006,21 +1021,24 @@
       <c r="S7" s="2">
         <v>1200</v>
       </c>
-      <c r="T7" s="4" t="s">
+      <c r="T7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U7" s="4" t="s">
+      <c r="U7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="V7" s="4" t="s">
+      <c r="V7" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="W7" s="4" t="s">
+      <c r="W7" s="2" t="s">
         <v>45</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" xr:uid="{A7955606-C781-4543-8983-1153BDF84C66}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Release 1.2.2: skins, recompensas, seleccion de apariencia y perfil.
Sistema de skins PvE y en mazos, recompensas Parent[n], modales de apariencia en desafios/eventos/coop/crear mazo, busqueda en seleccion de cartas, modal de perfil y skins limitados al mazo guardado.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/asaltos.xlsx
+++ b/public/resources/asaltos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01B666A-F980-466C-9D4C-2F8072027561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61D75DAB-0559-4198-8E20-902E7BC61A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="61">
   <si>
     <t>asalto_ID</t>
   </si>
@@ -165,7 +165,49 @@
     <t>1</t>
   </si>
   <si>
-    <t>https://images-ext-1.discordapp.net/external/4KzH3137pygQQi3r1ftpAi2LL9alkwXhYMY0R5kb8jA/https/speedforce.org/wp-content/uploads/2011/07/sdcc-flashpoint.jpg</t>
+    <t>Cyborg[0]</t>
+  </si>
+  <si>
+    <t>Batman[1]</t>
+  </si>
+  <si>
+    <t>Aquaman[2]</t>
+  </si>
+  <si>
+    <t>Wonder Woman[3]</t>
+  </si>
+  <si>
+    <t>Element Woman</t>
+  </si>
+  <si>
+    <t>Captain Cold[4]</t>
+  </si>
+  <si>
+    <t>Enchantress[5]</t>
+  </si>
+  <si>
+    <t>Joker[6]</t>
+  </si>
+  <si>
+    <t>Reverse Flash</t>
+  </si>
+  <si>
+    <t>Flash</t>
+  </si>
+  <si>
+    <t>Captain Thunder</t>
+  </si>
+  <si>
+    <t>Paradox Demon</t>
+  </si>
+  <si>
+    <t>tablero_background_speedforce</t>
+  </si>
+  <si>
+    <t>El tejido del tiempo se fractura de golpe para dar paso a una realidad distópica y devastada, donde Atlantis y Temiscira desatan una guerra mundial implacable; ahora, atrapado en el epicentro de un cataclismo temporal sin héroes, tu única opción de supervivencia es alterar el destino, desplegar una resistencia desesperada en combates tácticos por turnos y reescribir la historia antes de que el flashpoint original consuma el universo y borre la última línea temporal para siempre.</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/xqVnt8hX/Flashpoint.jpg</t>
   </si>
 </sst>
 </file>
@@ -539,6 +581,8 @@
     <col min="2" max="3" width="15" customWidth="1"/>
     <col min="4" max="5" width="17.85546875" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="16.140625" bestFit="1" customWidth="1"/>
@@ -695,52 +739,52 @@
         <v>34</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="2">
+        <v>6</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" s="2">
-        <v>7</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>25</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="S3" s="2">
         <v>1200</v>
@@ -1036,9 +1080,6 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" xr:uid="{A7955606-C781-4543-8983-1153BDF84C66}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add episodios mode with cutscenes, timeline combat, and hub integration.
Introduce episodios view (3D carousel), episodio engine (cutscene/combat/rewards), isolated ES_MODO_EPISODIO battle flow with catalog stat scaling, vistaJuego episodios panel with 2D preview carousel, and Centro de Operaciones layout updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/asaltos.xlsx
+++ b/public/resources/asaltos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61D75DAB-0559-4198-8E20-902E7BC61A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B363560D-3703-47B7-97C9-AAE432A234D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -195,9 +195,6 @@
     <t>Flash</t>
   </si>
   <si>
-    <t>Captain Thunder</t>
-  </si>
-  <si>
     <t>Paradox Demon</t>
   </si>
   <si>
@@ -208,6 +205,9 @@
   </si>
   <si>
     <t>https://i.ibb.co/xqVnt8hX/Flashpoint.jpg</t>
+  </si>
+  <si>
+    <t>Shazam[7]</t>
   </si>
 </sst>
 </file>
@@ -582,6 +582,7 @@
     <col min="4" max="5" width="17.85546875" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11" customWidth="1"/>
     <col min="17" max="17" width="15" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="15.5703125" bestFit="1" customWidth="1"/>
@@ -739,10 +740,10 @@
         <v>34</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E3" s="2">
         <v>6</v>
@@ -778,13 +779,13 @@
         <v>55</v>
       </c>
       <c r="P3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="R3" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="S3" s="2">
         <v>1200</v>

</xml_diff>